<commit_message>
fix in Excel template
</commit_message>
<xml_diff>
--- a/backend/templates/LeadImport_template.xlsx
+++ b/backend/templates/LeadImport_template.xlsx
@@ -928,7 +928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.88671875" defaultRowHeight="12" customHeight="1"/>
   <cols>
     <col width="11.109375" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -947,7 +947,7 @@
     <col width="21.109375" customWidth="1" style="2" min="14" max="14"/>
     <col width="23.88671875" customWidth="1" style="2" min="15" max="15"/>
     <col width="35.5546875" customWidth="1" style="2" min="16" max="16"/>
-    <col width="8.88671875" customWidth="1" style="2" min="17" max="16384"/>
+    <col width="35.5546875" customWidth="1" style="2" min="17" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.6" customHeight="1">
@@ -1029,6 +1029,11 @@
       <c r="P1" s="2" t="inlineStr">
         <is>
           <t>Source Detail</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>Industry_type</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1114,7 +1119,6 @@
           <t>company_name</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>Extracted company name.</t>
@@ -1127,8 +1131,6 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>Marketing-owned; left blank unless Marketing fills it in by hand.</t>
@@ -1146,8 +1148,6 @@
           <t>contact_person</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1160,8 +1160,6 @@
           <t>designation</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1174,8 +1172,6 @@
           <t>phone</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1188,8 +1184,6 @@
           <t>email</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1202,8 +1196,6 @@
           <t>address</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1216,8 +1208,6 @@
           <t>city</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1230,8 +1220,6 @@
           <t>gst</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1244,8 +1232,6 @@
           <t>turnover</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1258,8 +1244,6 @@
           <t>remarks</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1267,8 +1251,6 @@
           <t>Stage</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>Marketing-owned pipeline stage; left blank.</t>
@@ -1281,8 +1263,6 @@
           <t>Incharge</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>Marketing-owned; left blank.</t>
@@ -1295,8 +1275,6 @@
           <t>Alloted To</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>Marketing-owned; left blank.</t>
@@ -1309,11 +1287,26 @@
           <t>Source Detail</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>Marketing-owned; left blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Industry_type</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>industry</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Industry from public."TLead".industry_type.</t>
         </is>
       </c>
     </row>

</xml_diff>